<commit_message>
unit conversion bugs and other bugs
</commit_message>
<xml_diff>
--- a/config_data/units_mapping_x2x.xlsx
+++ b/config_data/units_mapping_x2x.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="31">
   <si>
     <t>%</t>
   </si>
@@ -51,64 +51,67 @@
     <t>MWh</t>
   </si>
   <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>kg</t>
+  </si>
+  <si>
+    <t>kg/MWh</t>
+  </si>
+  <si>
+    <t>kg/t</t>
+  </si>
+  <si>
+    <t>percent</t>
+  </si>
+  <si>
+    <t>t</t>
+  </si>
+  <si>
+    <t>€/MW</t>
+  </si>
+  <si>
+    <t>€/MWh</t>
+  </si>
+  <si>
+    <t>€/t</t>
+  </si>
+  <si>
+    <t>MEUR/GW</t>
+  </si>
+  <si>
+    <t>MEUR/(GW*a)</t>
+  </si>
+  <si>
+    <t>MEUR/GWh</t>
+  </si>
+  <si>
+    <t>GW</t>
+  </si>
+  <si>
+    <t>Kt/PJ</t>
+  </si>
+  <si>
+    <t>Kt/Mt</t>
+  </si>
+  <si>
+    <t>GWh</t>
+  </si>
+  <si>
+    <t>Source_Unit</t>
+  </si>
+  <si>
+    <t>Desired_unit</t>
+  </si>
+  <si>
+    <t>EUR/MW/a</t>
+  </si>
+  <si>
+    <t>€/MW*a</t>
+  </si>
+  <si>
     <t>MWh/MWh</t>
-  </si>
-  <si>
-    <t>a</t>
-  </si>
-  <si>
-    <t>kg</t>
-  </si>
-  <si>
-    <t>kg/MWh</t>
-  </si>
-  <si>
-    <t>kg/t</t>
-  </si>
-  <si>
-    <t>percent</t>
-  </si>
-  <si>
-    <t>t</t>
-  </si>
-  <si>
-    <t>€/MW</t>
-  </si>
-  <si>
-    <t>€/MWh</t>
-  </si>
-  <si>
-    <t>€/t</t>
-  </si>
-  <si>
-    <t>MEUR/GW</t>
-  </si>
-  <si>
-    <t>MEUR/(GW*a)</t>
-  </si>
-  <si>
-    <t>MEUR/GWh</t>
-  </si>
-  <si>
-    <t>GW</t>
-  </si>
-  <si>
-    <t>GWh/GWh</t>
-  </si>
-  <si>
-    <t>Kt/PJ</t>
-  </si>
-  <si>
-    <t>Kt/Mt</t>
-  </si>
-  <si>
-    <t>GWh</t>
-  </si>
-  <si>
-    <t>Source_Unit</t>
-  </si>
-  <si>
-    <t>Desired_unit</t>
   </si>
 </sst>
 </file>
@@ -129,7 +132,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -138,7 +141,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.39997558519241921"/>
+        <fgColor theme="9" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -170,12 +179,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -478,7 +489,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
@@ -487,174 +498,188 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="B4" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B5" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" t="s">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>1</v>
-      </c>
-      <c r="B10" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B12" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" t="s">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>12</v>
-      </c>
-      <c r="B13" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14" t="s">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B21" s="3"/>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B15" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>7</v>
-      </c>
-      <c r="B16" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>8</v>
-      </c>
-      <c r="B17" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>9</v>
-      </c>
-      <c r="B18" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>10</v>
-      </c>
-      <c r="B19" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+      <c r="B22" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B23" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>16</v>
-      </c>
-      <c r="B21" t="s">
-        <v>16</v>
-      </c>
-    </row>
   </sheetData>
-  <sortState ref="A2:B21">
+  <sortState ref="A2:B23">
     <sortCondition ref="A1"/>
   </sortState>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update units mapping and output data files
</commit_message>
<xml_diff>
--- a/config_data/units_mapping_x2x.xlsx
+++ b/config_data/units_mapping_x2x.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="32">
   <si>
     <t>%</t>
   </si>
@@ -112,6 +112,9 @@
   </si>
   <si>
     <t>MWh/MWh</t>
+  </si>
+  <si>
+    <t>MEUR/PJ</t>
   </si>
 </sst>
 </file>
@@ -601,11 +604,11 @@
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>21</v>
+      <c r="B14" s="3" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
pow_biogas_prod_de added to the process group and EUR/MW is added to unit mapping
</commit_message>
<xml_diff>
--- a/config_data/units_mapping_x2x.xlsx
+++ b/config_data/units_mapping_x2x.xlsx
@@ -1,25 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20395"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Xchange\Studis\Apath\HiWi Project\config_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\00_ESA\641_SEDOS BMWi\04-Arbeitspakete\AP9-Modellierung\data_adapter_TIMES\data_adapter_times_x2x\data_adapter_times\config_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6F5F778-EAA1-4EE0-9C33-96F6487F89E2}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6345"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6350" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Unique Units" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="33">
   <si>
     <t>%</t>
   </si>
@@ -115,12 +116,15 @@
   </si>
   <si>
     <t>MEUR/PJ</t>
+  </si>
+  <si>
+    <t>EUR/(MW*a)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -182,7 +186,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -190,9 +194,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -491,15 +496,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B24"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.7109375" customWidth="1"/>
+    <col min="1" max="1" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>26</v>
       </c>
@@ -507,7 +512,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -515,7 +520,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>16</v>
       </c>
@@ -523,7 +528,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
         <v>29</v>
       </c>
@@ -531,158 +536,166 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B6" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B7" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B8" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B9" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B10" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B11" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B12" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
         <v>2</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
-        <v>28</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A14" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A15" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B15" s="3" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A16" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B16" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B17" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B18" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A19" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B19" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B20" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B21" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B21" s="3"/>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
+      <c r="B22" s="3"/>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B23" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B24" s="2" t="s">
         <v>15</v>
       </c>
     </row>
   </sheetData>
-  <sortState ref="A2:B23">
+  <sortState ref="A2:B24">
     <sortCondition ref="A1"/>
   </sortState>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update configuration and output files: modify units mapping
</commit_message>
<xml_diff>
--- a/config_data/units_mapping_x2x.xlsx
+++ b/config_data/units_mapping_x2x.xlsx
@@ -1,25 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20416"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Xchange\Studis\Apath\HiWi Project\config_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\00_ESA\641_SEDOS BMWi\04-Arbeitspakete\AP9-Modellierung\data_adapter_TIMES\data_adapter_times_x2x\data_adapter_times\config_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD4B62BB-D2DD-4E08-809C-E578FD81E8E7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6345"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6350" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Unique Units" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="36">
   <si>
     <t>%</t>
   </si>
@@ -90,12 +91,6 @@
     <t>GW</t>
   </si>
   <si>
-    <t>Kt/PJ</t>
-  </si>
-  <si>
-    <t>Kt/Mt</t>
-  </si>
-  <si>
     <t>GWh</t>
   </si>
   <si>
@@ -115,12 +110,30 @@
   </si>
   <si>
     <t>MEUR/PJ</t>
+  </si>
+  <si>
+    <t>EUR/(MW*a)</t>
+  </si>
+  <si>
+    <t>t/MWh</t>
+  </si>
+  <si>
+    <t>MWh/t</t>
+  </si>
+  <si>
+    <t>PJ/kt</t>
+  </si>
+  <si>
+    <t>kt/PJ</t>
+  </si>
+  <si>
+    <t>kt/Mt</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -135,7 +148,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -151,6 +164,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -182,7 +201,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -190,9 +209,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -491,23 +512,23 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.7109375" customWidth="1"/>
+    <col min="1" max="1" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -515,7 +536,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>16</v>
       </c>
@@ -523,166 +544,190 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B6" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B7" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B8" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B9" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B10" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B11" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B12" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
         <v>2</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
-        <v>28</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A14" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A15" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B15" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A16" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="6" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B16" s="2" t="s">
+      <c r="B19" s="6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B21" s="3"/>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B23" s="3"/>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B24" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A25" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B25" s="2" t="s">
         <v>15</v>
       </c>
     </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>32</v>
+      </c>
+      <c r="B26" t="s">
+        <v>33</v>
+      </c>
+    </row>
   </sheetData>
-  <sortState ref="A2:B23">
+  <sortState ref="A2:B25">
     <sortCondition ref="A1"/>
   </sortState>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update 'unit_mapping' and 'Modellstruktur'
</commit_message>
<xml_diff>
--- a/config_data/units_mapping_x2x.xlsx
+++ b/config_data/units_mapping_x2x.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\00_ESA\641_SEDOS BMWi\04-Arbeitspakete\AP9-Modellierung\data_adapter_TIMES\data_adapter_times_x2x\data_adapter_times\config_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD4B62BB-D2DD-4E08-809C-E578FD81E8E7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1144896F-B3F3-4AA0-AA45-2932331D8E8A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6350" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="37">
   <si>
     <t>%</t>
   </si>
@@ -128,6 +128,9 @@
   </si>
   <si>
     <t>kt/Mt</t>
+  </si>
+  <si>
+    <t>MEUR/Kt</t>
   </si>
 </sst>
 </file>
@@ -677,7 +680,7 @@
         <v>7</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>7</v>
+        <v>36</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Update 'unit_mapping_x2x' and 'Final Modellstruktur'
</commit_message>
<xml_diff>
--- a/config_data/units_mapping_x2x.xlsx
+++ b/config_data/units_mapping_x2x.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\00_ESA\641_SEDOS BMWi\04-Arbeitspakete\AP9-Modellierung\data_adapter_TIMES\data_adapter_times_x2x\data_adapter_times\config_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD4B62BB-D2DD-4E08-809C-E578FD81E8E7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1144896F-B3F3-4AA0-AA45-2932331D8E8A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6350" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="37">
   <si>
     <t>%</t>
   </si>
@@ -128,6 +128,9 @@
   </si>
   <si>
     <t>kt/Mt</t>
+  </si>
+  <si>
+    <t>MEUR/Kt</t>
   </si>
 </sst>
 </file>
@@ -677,7 +680,7 @@
         <v>7</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>7</v>
+        <v>36</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">

</xml_diff>